<commit_message>
doc_url and dates attribute on archive pages; template updates
</commit_message>
<xml_diff>
--- a/resources/xlsx_templates/archive.xlsx
+++ b/resources/xlsx_templates/archive.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10413"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jbrandt/code/birddog/resources/xlsx_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEAE3FB1-53C9-924E-9BDB-F3404BADF46C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE598789-83F8-F444-8C7D-09BD3227D55D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10880" yWindow="9920" windowWidth="51660" windowHeight="12440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29120" yWindow="3640" windowWidth="34220" windowHeight="13100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="{id}" sheetId="2" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="41">
   <si>
     <t>source:</t>
   </si>
@@ -41,9 +41,6 @@
     <t>Archive link(s):</t>
   </si>
   <si>
-    <t>xxxxxxxxx</t>
-  </si>
-  <si>
     <t>TOTALS:</t>
   </si>
   <si>
@@ -153,6 +150,12 @@
   </si>
   <si>
     <t>{description}</t>
+  </si>
+  <si>
+    <t>{doc_url:doc_link}</t>
+  </si>
+  <si>
+    <t>{edit:nonexistent}</t>
   </si>
 </sst>
 </file>
@@ -162,7 +165,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000%"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -236,12 +239,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -295,14 +292,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
-      <sz val="11"/>
-      <color theme="1" tint="0.499984740745262"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="15"/>
       <color rgb="FF000000"/>
@@ -323,8 +312,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -409,12 +406,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFFF2CC"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -510,76 +501,76 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -588,15 +579,14 @@
     <xf numFmtId="0" fontId="7" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -620,7 +610,7 @@
     <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -629,7 +619,7 @@
     <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -638,51 +628,50 @@
     <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="12" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -907,49 +896,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" ht="28">
-      <c r="A1" s="42" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="44" t="s">
+      <c r="A1" s="41" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="42"/>
+      <c r="C1" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" s="44"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="48" t="s">
         <v>34</v>
       </c>
-      <c r="D1" s="45"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="47"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="42"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="49" t="s">
+      <c r="L1" s="49"/>
+      <c r="M1" s="48" t="s">
         <v>35</v>
       </c>
-      <c r="L1" s="50"/>
-      <c r="M1" s="49" t="s">
-        <v>36</v>
-      </c>
-      <c r="N1" s="51" t="s">
-        <v>33</v>
-      </c>
-      <c r="O1" s="38" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q1" s="47"/>
-      <c r="R1" s="45"/>
-      <c r="S1" s="45"/>
-      <c r="T1" s="45"/>
-      <c r="U1" s="45"/>
-      <c r="V1" s="45"/>
-      <c r="W1" s="45"/>
-      <c r="X1" s="45"/>
-      <c r="Y1" s="45"/>
-      <c r="Z1" s="52"/>
-      <c r="AA1" s="45"/>
-      <c r="AB1" s="45"/>
+      <c r="N1" s="50" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q1" s="46"/>
+      <c r="R1" s="44"/>
+      <c r="S1" s="44"/>
+      <c r="T1" s="44"/>
+      <c r="U1" s="44"/>
+      <c r="V1" s="44"/>
+      <c r="W1" s="44"/>
+      <c r="X1" s="44"/>
+      <c r="Y1" s="44"/>
+      <c r="Z1" s="51"/>
+      <c r="AA1" s="44"/>
+      <c r="AB1" s="44"/>
     </row>
     <row r="2" spans="1:28" ht="19">
       <c r="A2" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="3"/>
@@ -961,12 +947,9 @@
       <c r="I2" s="1"/>
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
-      <c r="L2" s="53"/>
-      <c r="M2" s="54"/>
+      <c r="L2" s="52"/>
+      <c r="M2" s="53"/>
       <c r="N2" s="1"/>
-      <c r="O2" s="39" t="s">
-        <v>27</v>
-      </c>
       <c r="Q2" s="4"/>
       <c r="R2" s="2"/>
       <c r="S2" s="2"/>
@@ -976,7 +959,7 @@
       <c r="W2" s="2"/>
       <c r="X2" s="2"/>
       <c r="Y2" s="2"/>
-      <c r="Z2" s="55"/>
+      <c r="Z2" s="54"/>
       <c r="AA2" s="2"/>
       <c r="AB2" s="2"/>
     </row>
@@ -987,21 +970,18 @@
         <v>0</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E3" s="6"/>
       <c r="F3" s="8"/>
       <c r="G3" s="9"/>
       <c r="H3" s="6"/>
       <c r="I3" s="9"/>
-      <c r="J3" s="56"/>
-      <c r="K3" s="56"/>
-      <c r="L3" s="56"/>
-      <c r="M3" s="57"/>
-      <c r="N3" s="57"/>
-      <c r="O3" s="40" t="s">
-        <v>28</v>
-      </c>
+      <c r="J3" s="55"/>
+      <c r="K3" s="55"/>
+      <c r="L3" s="55"/>
+      <c r="M3" s="56"/>
+      <c r="N3" s="56"/>
       <c r="P3" s="7"/>
       <c r="Q3" s="7"/>
       <c r="R3" s="7"/>
@@ -1020,8 +1000,8 @@
       <c r="A4" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="58" t="s">
-        <v>2</v>
+      <c r="B4" s="7" t="s">
+        <v>39</v>
       </c>
       <c r="C4" s="11"/>
       <c r="D4" s="12"/>
@@ -1035,20 +1015,17 @@
       <c r="L4" s="13"/>
       <c r="M4" s="13"/>
       <c r="N4" s="12"/>
-      <c r="O4" s="41" t="s">
-        <v>29</v>
-      </c>
       <c r="P4" s="13"/>
       <c r="Q4" s="13"/>
-      <c r="R4" s="59"/>
-      <c r="S4" s="59"/>
-      <c r="T4" s="59"/>
-      <c r="U4" s="59"/>
-      <c r="V4" s="59"/>
-      <c r="W4" s="59"/>
-      <c r="X4" s="59"/>
-      <c r="Y4" s="59"/>
-      <c r="Z4" s="60"/>
+      <c r="R4" s="57"/>
+      <c r="S4" s="57"/>
+      <c r="T4" s="57"/>
+      <c r="U4" s="57"/>
+      <c r="V4" s="57"/>
+      <c r="W4" s="57"/>
+      <c r="X4" s="57"/>
+      <c r="Y4" s="57"/>
+      <c r="Z4" s="58"/>
       <c r="AA4" s="7"/>
       <c r="AB4" s="7"/>
     </row>
@@ -1057,37 +1034,37 @@
       <c r="B5" s="15"/>
       <c r="C5" s="16"/>
       <c r="D5" s="17" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H5" s="18" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I5" s="19" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J5" s="19" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="L5" s="19" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="M5" s="20" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="N5" s="21" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O5" s="11"/>
       <c r="P5" s="15"/>
@@ -1105,86 +1082,86 @@
       <c r="AB5" s="15"/>
     </row>
     <row r="6" spans="1:28" ht="48">
-      <c r="A6" s="61" t="s">
+      <c r="A6" s="59" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="60" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="62" t="s">
+      <c r="C6" s="61" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="63" t="s">
+      <c r="D6" s="59" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="61" t="s">
+      <c r="E6" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="22" t="s">
+      <c r="F6" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="F6" s="22" t="s">
+      <c r="G6" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="G6" s="22" t="s">
+      <c r="H6" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="H6" s="22" t="s">
+      <c r="I6" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="I6" s="23" t="s">
+      <c r="J6" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="J6" s="23" t="s">
+      <c r="K6" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="K6" s="23" t="s">
+      <c r="L6" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="L6" s="23" t="s">
+      <c r="M6" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="M6" s="24" t="s">
+      <c r="N6" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="N6" s="25" t="s">
+      <c r="O6" s="62" t="s">
         <v>17</v>
       </c>
-      <c r="O6" s="64" t="s">
-        <v>18</v>
-      </c>
-      <c r="P6" s="65"/>
-      <c r="Q6" s="65"/>
+      <c r="P6" s="63"/>
+      <c r="Q6" s="63"/>
       <c r="R6" s="26"/>
-      <c r="S6" s="65"/>
-      <c r="T6" s="65"/>
-      <c r="U6" s="65"/>
-      <c r="V6" s="65"/>
-      <c r="W6" s="65"/>
-      <c r="X6" s="65"/>
-      <c r="Y6" s="65"/>
-      <c r="Z6" s="65"/>
-      <c r="AA6" s="65"/>
-      <c r="AB6" s="65"/>
+      <c r="S6" s="63"/>
+      <c r="T6" s="63"/>
+      <c r="U6" s="63"/>
+      <c r="V6" s="63"/>
+      <c r="W6" s="63"/>
+      <c r="X6" s="63"/>
+      <c r="Y6" s="63"/>
+      <c r="Z6" s="63"/>
+      <c r="AA6" s="63"/>
+      <c r="AB6" s="63"/>
     </row>
     <row r="7" spans="1:28">
       <c r="A7" s="27" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B7" s="28"/>
       <c r="C7" s="29"/>
       <c r="D7" s="30"/>
-      <c r="E7" s="66"/>
-      <c r="F7" s="66"/>
-      <c r="G7" s="66"/>
-      <c r="H7" s="66"/>
-      <c r="I7" s="66"/>
-      <c r="J7" s="66"/>
-      <c r="K7" s="66"/>
-      <c r="L7" s="66"/>
+      <c r="E7" s="64"/>
+      <c r="F7" s="64"/>
+      <c r="G7" s="64"/>
+      <c r="H7" s="64"/>
+      <c r="I7" s="64"/>
+      <c r="J7" s="64"/>
+      <c r="K7" s="64"/>
+      <c r="L7" s="64"/>
       <c r="M7" s="31"/>
       <c r="N7" s="31"/>
       <c r="O7" s="31"/>
       <c r="P7" s="15"/>
       <c r="Q7" s="15"/>
-      <c r="R7" s="67"/>
+      <c r="R7" s="65"/>
       <c r="S7" s="15"/>
       <c r="T7" s="15"/>
       <c r="U7" s="15"/>
@@ -1198,53 +1175,53 @@
     </row>
     <row r="8" spans="1:28" ht="16">
       <c r="A8" s="32" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="33" t="s">
+      <c r="C8" s="66" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="68" t="s">
-        <v>32</v>
-      </c>
-      <c r="D8" s="69" t="s">
-        <v>22</v>
-      </c>
-      <c r="E8" s="70" t="s">
-        <v>22</v>
-      </c>
-      <c r="F8" s="70" t="s">
-        <v>22</v>
-      </c>
-      <c r="G8" s="70" t="s">
-        <v>22</v>
-      </c>
-      <c r="H8" s="70" t="s">
-        <v>22</v>
-      </c>
-      <c r="I8" s="70" t="s">
-        <v>22</v>
-      </c>
-      <c r="J8" s="70" t="s">
-        <v>22</v>
-      </c>
-      <c r="K8" s="70" t="s">
-        <v>22</v>
-      </c>
-      <c r="L8" s="70" t="s">
-        <v>22</v>
-      </c>
-      <c r="M8" s="70" t="s">
-        <v>22</v>
-      </c>
-      <c r="N8" s="70" t="s">
-        <v>22</v>
-      </c>
-      <c r="O8" s="71" t="s">
-        <v>22</v>
+      <c r="D8" s="67" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" s="68" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="68" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" s="68" t="s">
+        <v>21</v>
+      </c>
+      <c r="H8" s="68" t="s">
+        <v>21</v>
+      </c>
+      <c r="I8" s="68" t="s">
+        <v>21</v>
+      </c>
+      <c r="J8" s="68" t="s">
+        <v>21</v>
+      </c>
+      <c r="K8" s="68" t="s">
+        <v>21</v>
+      </c>
+      <c r="L8" s="68" t="s">
+        <v>21</v>
+      </c>
+      <c r="M8" s="68" t="s">
+        <v>21</v>
+      </c>
+      <c r="N8" s="68" t="s">
+        <v>21</v>
+      </c>
+      <c r="O8" s="69" t="s">
+        <v>21</v>
       </c>
       <c r="P8" s="15"/>
       <c r="Q8" s="15"/>
-      <c r="R8" s="67"/>
+      <c r="R8" s="65"/>
       <c r="S8" s="15"/>
       <c r="T8" s="15"/>
       <c r="U8" s="15"/>
@@ -1288,10 +1265,10 @@
     </row>
     <row r="10" spans="1:28">
       <c r="A10" s="36" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C10" s="15"/>
       <c r="D10" s="15"/>
@@ -1303,10 +1280,10 @@
       <c r="J10" s="15"/>
       <c r="K10" s="15"/>
       <c r="L10" s="37" t="s">
-        <v>21</v>
-      </c>
-      <c r="M10" s="72" t="s">
-        <v>25</v>
+        <v>20</v>
+      </c>
+      <c r="M10" s="70" t="s">
+        <v>24</v>
       </c>
       <c r="N10" s="15"/>
       <c r="O10" s="15"/>
@@ -1369,7 +1346,9 @@
       <c r="L12" s="16"/>
       <c r="M12" s="16"/>
       <c r="N12" s="16"/>
-      <c r="O12" s="15"/>
+      <c r="O12" s="38" t="s">
+        <v>25</v>
+      </c>
       <c r="P12" s="15"/>
       <c r="Q12" s="15"/>
       <c r="R12" s="15"/>
@@ -1399,7 +1378,9 @@
       <c r="L13" s="16"/>
       <c r="M13" s="16"/>
       <c r="N13" s="16"/>
-      <c r="O13" s="15"/>
+      <c r="O13" s="39" t="s">
+        <v>26</v>
+      </c>
       <c r="P13" s="15"/>
       <c r="Q13" s="15"/>
       <c r="R13" s="15"/>
@@ -1429,7 +1410,9 @@
       <c r="L14" s="16"/>
       <c r="M14" s="16"/>
       <c r="N14" s="16"/>
-      <c r="O14" s="15"/>
+      <c r="O14" s="40" t="s">
+        <v>27</v>
+      </c>
       <c r="P14" s="15"/>
       <c r="Q14" s="15"/>
       <c r="R14" s="15"/>
@@ -1459,7 +1442,9 @@
       <c r="L15" s="16"/>
       <c r="M15" s="16"/>
       <c r="N15" s="16"/>
-      <c r="O15" s="15"/>
+      <c r="O15" s="72" t="s">
+        <v>28</v>
+      </c>
       <c r="P15" s="15"/>
       <c r="Q15" s="15"/>
       <c r="R15" s="15"/>
@@ -1489,7 +1474,9 @@
       <c r="L16" s="16"/>
       <c r="M16" s="16"/>
       <c r="N16" s="16"/>
-      <c r="O16" s="15"/>
+      <c r="O16" s="71" t="s">
+        <v>40</v>
+      </c>
       <c r="P16" s="15"/>
       <c r="Q16" s="15"/>
       <c r="R16" s="15"/>

</xml_diff>

<commit_message>
fix #46: template changes
</commit_message>
<xml_diff>
--- a/resources/xlsx_templates/archive.xlsx
+++ b/resources/xlsx_templates/archive.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jbrandt/code/birddog/resources/xlsx_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE598789-83F8-F444-8C7D-09BD3227D55D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2626DC73-F4B7-464C-93C1-4A0481258566}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="29120" yWindow="3640" windowWidth="34220" windowHeight="13100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="50">
   <si>
     <t>source:</t>
   </si>
@@ -101,12 +101,6 @@
     <t>{empty}</t>
   </si>
   <si>
-    <t>=SUM(__COL__)</t>
-  </si>
-  <si>
-    <t>=ROWS(__COL__)</t>
-  </si>
-  <si>
     <t>=(F$5+J$5)/M$5</t>
   </si>
   <si>
@@ -156,6 +150,39 @@
   </si>
   <si>
     <t>{edit:nonexistent}</t>
+  </si>
+  <si>
+    <t>=ROWS($A$__FIRST__:$A__LAST__)</t>
+  </si>
+  <si>
+    <t>=SUM(E$__FIRST__:E__LAST__)</t>
+  </si>
+  <si>
+    <t>=SUM(F$__FIRST__:F__LAST__)</t>
+  </si>
+  <si>
+    <t>=SUM(G$__FIRST__:G__LAST__)</t>
+  </si>
+  <si>
+    <t>=SUM(H$__FIRST__:H__LAST__)</t>
+  </si>
+  <si>
+    <t>=SUM(I$__FIRST__:I__LAST__)</t>
+  </si>
+  <si>
+    <t>=SUM(J$__FIRST__:J__LAST__)</t>
+  </si>
+  <si>
+    <t>=SUM(K$__FIRST__:K__LAST__)</t>
+  </si>
+  <si>
+    <t>=SUM(L$__FIRST__:L__LAST__)</t>
+  </si>
+  <si>
+    <t>=SUM(M$__FIRST__:M__LAST__)</t>
+  </si>
+  <si>
+    <t>=SUM(N$__FIRST__:N__LAST__)</t>
   </si>
 </sst>
 </file>
@@ -897,11 +924,11 @@
   <sheetData>
     <row r="1" spans="1:28" ht="28">
       <c r="A1" s="41" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B1" s="42"/>
       <c r="C1" s="43" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D1" s="44"/>
       <c r="E1" s="45"/>
@@ -911,14 +938,14 @@
       <c r="I1" s="41"/>
       <c r="J1" s="45"/>
       <c r="K1" s="48" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="L1" s="49"/>
       <c r="M1" s="48" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="N1" s="50" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="Q1" s="46"/>
       <c r="R1" s="44"/>
@@ -935,7 +962,7 @@
     </row>
     <row r="2" spans="1:28" ht="19">
       <c r="A2" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="3"/>
@@ -970,7 +997,7 @@
         <v>0</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E3" s="6"/>
       <c r="F3" s="8"/>
@@ -1001,7 +1028,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C4" s="11"/>
       <c r="D4" s="12"/>
@@ -1037,34 +1064,34 @@
         <v>2</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="H5" s="18" t="s">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="I5" s="19" t="s">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="J5" s="19" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="L5" s="19" t="s">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="M5" s="20" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="N5" s="21" t="s">
-        <v>22</v>
+        <v>49</v>
       </c>
       <c r="O5" s="11"/>
       <c r="P5" s="15"/>
@@ -1175,13 +1202,13 @@
     </row>
     <row r="8" spans="1:28" ht="16">
       <c r="A8" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="33" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="66" t="s">
         <v>29</v>
-      </c>
-      <c r="B8" s="33" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" s="66" t="s">
-        <v>31</v>
       </c>
       <c r="D8" s="67" t="s">
         <v>21</v>
@@ -1265,7 +1292,7 @@
     </row>
     <row r="10" spans="1:28">
       <c r="A10" s="36" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="B10" s="15" t="s">
         <v>19</v>
@@ -1283,7 +1310,7 @@
         <v>20</v>
       </c>
       <c r="M10" s="70" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="N10" s="15"/>
       <c r="O10" s="15"/>
@@ -1347,7 +1374,7 @@
       <c r="M12" s="16"/>
       <c r="N12" s="16"/>
       <c r="O12" s="38" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="P12" s="15"/>
       <c r="Q12" s="15"/>
@@ -1379,7 +1406,7 @@
       <c r="M13" s="16"/>
       <c r="N13" s="16"/>
       <c r="O13" s="39" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="P13" s="15"/>
       <c r="Q13" s="15"/>
@@ -1411,7 +1438,7 @@
       <c r="M14" s="16"/>
       <c r="N14" s="16"/>
       <c r="O14" s="40" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="P14" s="15"/>
       <c r="Q14" s="15"/>
@@ -1443,7 +1470,7 @@
       <c r="M15" s="16"/>
       <c r="N15" s="16"/>
       <c r="O15" s="72" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="P15" s="15"/>
       <c r="Q15" s="15"/>
@@ -1475,7 +1502,7 @@
       <c r="M16" s="16"/>
       <c r="N16" s="16"/>
       <c r="O16" s="71" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="P16" s="15"/>
       <c r="Q16" s="15"/>

</xml_diff>